<commit_message>
Polish design workbook formatting
</commit_message>
<xml_diff>
--- a/docs/design/01_基本設計書_HackerLake.xlsx
+++ b/docs/design/01_基本設計書_HackerLake.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phrx4\hackerlake\docs\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E11AC9A1-3B12-45D8-BA8F-9DBC280E4106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4E1DAAC-C810-436E-9A42-3C1E2E9A3772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{C6E4A6BA-C340-4995-8641-72806C7AE8B0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{572EB544-28CB-4844-AFF5-1EA35AAF9571}"/>
   </bookViews>
   <sheets>
     <sheet name="表紙" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,20 @@
     <sheet name="非機能要件" sheetId="5" r:id="rId5"/>
     <sheet name="トレーサビリティ" sheetId="6" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">トレーサビリティ!$A$3:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">改訂履歴!$A$3:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">機能一覧!$A$3:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">非機能要件!$A$3:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">表紙!$A$3:$H$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">要件一覧!$A$3:$H$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">トレーサビリティ!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">改訂履歴!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">機能一覧!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">非機能要件!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">表紙!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">要件一覧!$1:$3</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -609,7 +623,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -636,15 +650,21 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="游ゴシック"/>
+      <name val="Yu Gothic"/>
       <family val="3"/>
       <charset val="128"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -660,6 +680,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF006080"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7FAFC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -693,7 +719,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -701,12 +727,18 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1022,18 +1054,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD815368-B010-4FD7-8B48-81E04B9374F0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82A81DD2-E66C-4D05-874F-43E48F529E9F}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="16.625" customWidth="1"/>
-    <col min="2" max="2" width="24.625" customWidth="1"/>
-    <col min="3" max="3" width="34.625" customWidth="1"/>
-    <col min="4" max="5" width="42.625" customWidth="1"/>
-    <col min="6" max="8" width="28.625" customWidth="1"/>
+    <col min="1" max="1" width="15.625" customWidth="1"/>
+    <col min="2" max="2" width="22.625" customWidth="1"/>
+    <col min="3" max="3" width="36.625" customWidth="1"/>
+    <col min="4" max="5" width="46.625" customWidth="1"/>
+    <col min="6" max="7" width="28.625" customWidth="1"/>
+    <col min="8" max="8" width="24.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1045,7 +1081,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="32.1" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1071,7 +1107,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
@@ -1089,33 +1125,33 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="5">
         <v>46186</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>20</v>
       </c>
@@ -1142,27 +1178,33 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:H6" xr:uid="{82A81DD2-E66C-4D05-874F-43E48F529E9F}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.3" right="0.3" top="0.44999999999999996" bottom="0.44999999999999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BF284D5-9596-490F-A10F-9DFE08C54C01}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3C347AB-489F-4854-B92C-B3A449CB95BC}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="16.625" customWidth="1"/>
-    <col min="2" max="2" width="24.625" customWidth="1"/>
-    <col min="3" max="3" width="34.625" customWidth="1"/>
-    <col min="4" max="5" width="42.625" customWidth="1"/>
-    <col min="6" max="8" width="28.625" customWidth="1"/>
+    <col min="1" max="1" width="15.625" customWidth="1"/>
+    <col min="2" max="2" width="22.625" customWidth="1"/>
+    <col min="3" max="3" width="36.625" customWidth="1"/>
+    <col min="4" max="5" width="46.625" customWidth="1"/>
+    <col min="6" max="7" width="28.625" customWidth="1"/>
+    <col min="8" max="8" width="24.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1174,7 +1216,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="32.1" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
@@ -1200,11 +1242,11 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A4" s="3">
         <v>1</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="6">
         <v>46186</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -1222,50 +1264,56 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3">
+    <row r="5" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A5" s="4">
         <v>1.1000000000000001</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
     </row>
   </sheetData>
+  <autoFilter ref="A3:H5" xr:uid="{C3C347AB-489F-4854-B92C-B3A449CB95BC}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.3" right="0.3" top="0.44999999999999996" bottom="0.44999999999999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8EB4AB5-DA41-407C-AEEF-3FCC4D4AA302}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35961221-366F-4B10-B004-8B0DAEAAD689}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="16.625" customWidth="1"/>
-    <col min="2" max="2" width="24.625" customWidth="1"/>
-    <col min="3" max="3" width="34.625" customWidth="1"/>
-    <col min="4" max="5" width="42.625" customWidth="1"/>
-    <col min="6" max="8" width="28.625" customWidth="1"/>
+    <col min="1" max="1" width="15.625" customWidth="1"/>
+    <col min="2" max="2" width="22.625" customWidth="1"/>
+    <col min="3" max="3" width="36.625" customWidth="1"/>
+    <col min="4" max="5" width="46.625" customWidth="1"/>
+    <col min="6" max="7" width="28.625" customWidth="1"/>
+    <col min="8" max="8" width="24.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>43</v>
       </c>
@@ -1277,7 +1325,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="32.1" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>44</v>
       </c>
@@ -1303,7 +1351,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>52</v>
       </c>
@@ -1329,33 +1377,33 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A5" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>65</v>
       </c>
@@ -1381,33 +1429,33 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A7" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>77</v>
       </c>
@@ -1433,33 +1481,33 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A9" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>90</v>
       </c>
@@ -1486,27 +1534,33 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:H10" xr:uid="{35961221-366F-4B10-B004-8B0DAEAAD689}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.3" right="0.3" top="0.44999999999999996" bottom="0.44999999999999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC216123-93BD-4BE6-B7EE-8D27066A1479}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41FDBB58-0224-4386-9657-1BF7E1A0E8BD}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="16.625" customWidth="1"/>
-    <col min="2" max="2" width="24.625" customWidth="1"/>
-    <col min="3" max="3" width="34.625" customWidth="1"/>
-    <col min="4" max="5" width="42.625" customWidth="1"/>
-    <col min="6" max="8" width="28.625" customWidth="1"/>
+    <col min="1" max="1" width="15.625" customWidth="1"/>
+    <col min="2" max="2" width="22.625" customWidth="1"/>
+    <col min="3" max="3" width="36.625" customWidth="1"/>
+    <col min="4" max="5" width="46.625" customWidth="1"/>
+    <col min="6" max="7" width="28.625" customWidth="1"/>
+    <col min="8" max="8" width="24.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>97</v>
       </c>
@@ -1518,7 +1572,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="32.1" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>98</v>
       </c>
@@ -1544,7 +1598,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>57</v>
       </c>
@@ -1570,33 +1624,33 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A5" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>63</v>
       </c>
@@ -1622,33 +1676,33 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A7" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>121</v>
       </c>
@@ -1674,54 +1728,60 @@
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A9" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="4" t="s">
         <v>56</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:H9" xr:uid="{41FDBB58-0224-4386-9657-1BF7E1A0E8BD}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.3" right="0.3" top="0.44999999999999996" bottom="0.44999999999999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B3BEEE6-789F-4180-B207-814D097D9561}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CA88A0A-0E8C-4D6C-A353-67C4DDDCC353}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="16.625" customWidth="1"/>
-    <col min="2" max="2" width="24.625" customWidth="1"/>
-    <col min="3" max="3" width="34.625" customWidth="1"/>
-    <col min="4" max="5" width="42.625" customWidth="1"/>
-    <col min="6" max="8" width="28.625" customWidth="1"/>
+    <col min="1" max="1" width="15.625" customWidth="1"/>
+    <col min="2" max="2" width="22.625" customWidth="1"/>
+    <col min="3" max="3" width="36.625" customWidth="1"/>
+    <col min="4" max="5" width="46.625" customWidth="1"/>
+    <col min="6" max="7" width="28.625" customWidth="1"/>
+    <col min="8" max="8" width="24.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>133</v>
       </c>
@@ -1733,7 +1793,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="32.1" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>134</v>
       </c>
@@ -1759,7 +1819,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>137</v>
       </c>
@@ -1785,33 +1845,33 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A5" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>148</v>
       </c>
@@ -1837,33 +1897,33 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A7" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>157</v>
       </c>
@@ -1890,27 +1950,33 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:H8" xr:uid="{6CA88A0A-0E8C-4D6C-A353-67C4DDDCC353}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.3" right="0.3" top="0.44999999999999996" bottom="0.44999999999999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BF5B218-456C-43E4-B854-0BC7DD0E41E1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41289B1E-C9EA-4736-A4F9-74FBE288E5C8}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="16.625" customWidth="1"/>
-    <col min="2" max="2" width="24.625" customWidth="1"/>
-    <col min="3" max="3" width="34.625" customWidth="1"/>
-    <col min="4" max="5" width="42.625" customWidth="1"/>
-    <col min="6" max="8" width="28.625" customWidth="1"/>
+    <col min="1" max="1" width="15.625" customWidth="1"/>
+    <col min="2" max="2" width="22.625" customWidth="1"/>
+    <col min="3" max="3" width="36.625" customWidth="1"/>
+    <col min="4" max="5" width="46.625" customWidth="1"/>
+    <col min="6" max="7" width="28.625" customWidth="1"/>
+    <col min="8" max="8" width="24.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -1922,7 +1988,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="32.1" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>44</v>
       </c>
@@ -1948,7 +2014,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>52</v>
       </c>
@@ -1974,33 +2040,33 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A5" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>65</v>
       </c>
@@ -2026,33 +2092,33 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A7" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:8" ht="33.950000000000003" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>90</v>
       </c>
@@ -2079,10 +2145,12 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:H8" xr:uid="{41289B1E-C9EA-4736-A4F9-74FBE288E5C8}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.3" right="0.3" top="0.44999999999999996" bottom="0.44999999999999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>